<commit_message>
Atualização automática - 03/03/2026 09:06
</commit_message>
<xml_diff>
--- a/dados/01 a 15-02/PEDIDOS_DIA.xlsx
+++ b/dados/01 a 15-02/PEDIDOS_DIA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b754a023a117f00d/Documentos/python/Projetos/Dashboard_Sauipe/dados/01 a 15-02/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos_Python\Dashboard_Sauipe\dados\01 a 15-02\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{003BDE5D-5FAB-4209-8230-D2D00BA08D0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4FA3EF8-86E4-4C68-A663-D9553136A622}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{BAE7E909-A9ED-4488-BF07-0D01A6757217}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{BAE7E909-A9ED-4488-BF07-0D01A6757217}"/>
   </bookViews>
   <sheets>
     <sheet name="HISTOGRAMA" sheetId="1" r:id="rId1"/>
@@ -417,10 +417,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>